<commit_message>
updating notes on sus aspects of current implementation
</commit_message>
<xml_diff>
--- a/Overview_v0.xlsx
+++ b/Overview_v0.xlsx
@@ -3091,8 +3091,9 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Each region exposes trimesh submesh.volume and .area directly. The submeshes come from plane-slicing plus trimesh fill_holes (arm, leg, head) or boolean difference (trunk).
-Honest: fill_holes tries to cap the cut opening but does not guarantee a watertight mesh, so .volume is only meaningful when capping succeeds and can be wrong on complex or multi-loop cut boundaries. There is no explicit cap step or fixFaceOrientation equivalent like the MATLAB partial-volume routine, and .area includes any uncapped boundary.</t>
+          <t>Each region defines volume/surface_area properties, but they are effectively non-functional.
+Verified on man.obj: Arm and Trunk return self._trimesh.volume/.area and _trimesh is never assigned in src, so left arm, right arm and trunk all raise AttributeError. Leg and Head return self.mesh.volume/.area and run, but give NEGATIVE volumes (head ~ -9.8, each leg ~ -20.85), i.e. inverted/non-watertight results.
+Gap: no winding fix (no fixFaceOrientation equivalent) and no capping of the sliced openings, and the Arm/Trunk _trimesh reference is a latent bug. Nothing in body.py or main.py reads volume/area, so the breakage is currently silent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Python geometry benchmark reporting
</commit_message>
<xml_diff>
--- a/Overview_v0.xlsx
+++ b/Overview_v0.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATLAB" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TopoSort" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MATLAB" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Python" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TopoSort" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -74,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -97,6 +97,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2259,7 +2262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z38"/>
+  <dimension ref="A1:Z39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="31.75" customWidth="1" style="9" min="1" max="1"/>
@@ -2358,16 +2361,16 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Raw Vertices (v)</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Cleaning - &gt; Normalization -&gt; Axis Alignment
-1. Cleaning: Uses standard trimesh functions to fill holes, remove unreferenced vertices, and ensure face integrity.
-2. Normalization: The mesh is centered at the origin, and its vertex coordinates are scaled based on their standard deviation. This makes subsequent algorithms independent of the mesh's original scale and position. 
-3. Height Axis Alignment: It identifies the body's longest axis (X, Y, or Z) and rotates the mesh to align this primary axis with the Z-axis (height).
-4. Left-Right Axis Alignment: This is a complex heuristic. It creates a KD-Tree for fast spatial queries. It then samples points along two vertical lines at the mesh's outer extents (one on the X-min, one on the Y-min). It finds the nearest mesh vertices to these lines and calculates which set of vertices forms a "flatter" plane (i.e., which axis represents the front/back profile vs. the side profile). The flatter profile is determined to be the front/back, and the axes are swapped if necessary so that X corresponds to the left-right direction.</t>
+          <t>Raw Vertices (v), input units</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Cleaning -&gt; unit normalization -&gt; orientation -&gt; scale-aware geometry config.
+1. Body.__init__ loads the mesh, calls build_geometry_config(mesh, units), converts vertices to internal dm, and stores geometry_config in mesh.metadata.
+2. density_scale = median(edges_unique_length)*unit_to_internal / BASELINE_MEDIAN_EDGE_LENGTH. Slice widths and anatomical bands scale by this value.
+3. Mesh orientation then aligns z with height and x with left-right.
+Current: use --units dm for man.obj; use --units mm for scanner OBJ files and penn-mesh-2.obj.</t>
         </is>
       </c>
     </row>
@@ -2460,18 +2463,16 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Oriented Mesh</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>convexity_search: This is the primary measurement algorithm and the main computational bottleneck. It's an iterative search that moves up the body from below, analyzing the shape of horizontal cross-sections to find the point where the gap between the legs ends. 
-1. Find Start Point: It first casts a ray up the Z-axis from the bottom to find a starting point in the inseam area. 
-2. Iterative Slicing: It begins a loop, moving a search origin upwards in small, discrete steps. 
-3. Ray Casting &amp; Intersection: In each iteration, it casts a fan of 32 rays horizontally out from the origin. It finds all points where these rays intersect the mesh.
-4. Loop Creation: For each ray, it finds the outermost intersection point to define the body's perimeter at that slice. These points are then ordered by angle to form a 2D loop. 
-5. Convexity Analysis: It uses the shapely library to calculate the "convexity score" of this 2D loop (defined as Area / Convex Hull Area). A score near 1.0 indicates a convex shape (like the torso), while a lower score indicates a concave shape (the gap between the legs). 
-6. Termination: The algorithm stops and returns the center of the slice as the crotch point as soon as it finds a slice with a convexity score above a set threshold (e.g., &gt;0.95), signifying it has cleared the leg gap. If the threshold isn't met, it returns the point from the most convex slice it found.</t>
+          <t>Oriented Mesh, Feet, Section Loops</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>locate_crotch is staged rather than a single convexity stop.
+1. convexity_search gives an initial saddle estimate from upward horizontal ray fans.
+2. If (crotch_z-min_z)/height &lt; 0.40, maxmin_crotch_point raises to max_x min_z(column) between the feet.
+3. topology_crotch_point scans upward: first observe separate left/right leg loops; after merge, compute neck_ratio = y_span(x?0)/mean(y_span(side lobes)). Return the first merged central section crossing an adaptive percentile threshold.
+Purpose: reject underwear/contact bridges and raise to the pelvis/glute saddle when section topology supports it.</t>
         </is>
       </c>
     </row>
@@ -2493,11 +2494,10 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>_locate_armpits -&gt; _trace_hip_to_armpit (per side).
-1. From each hip, take vertices in an 8cm-wide lateral band (hip_x +/- 4cm) with z &gt;= hip_z.
-2. Sort by z and walk upward until the z-increase between successive points drops below 0.5cm; that stall is the armpit candidate (arm bends away from torso).
-3. Refine with convexity_search (32 rays) and snap to the nearest mesh vertex; on failure, fall back to the candidate.
-Honest: assumes arms-down A-pose and a clean lateral surface. The 8cm band and 0.5cm stall threshold are hard-coded for ~unit/metre scale and break on a T-pose or differently scaled mesh.</t>
+          <t>locate_armpits now uses candidate pooling plus bilateral scoring.
+Per side candidates: trace_hip_to_armpit, section_merge_armpit_candidates, section_gap_armpit, side_gap_armpit.
+Score = source weight + relative-height score + arm_support_score + arm_cut_viability_score. choose_armpit_pair penalizes left/right relative-height and z mismatch; rebalance_high_armpit lowers one-sided shoulder-cap choices.
+Current interpretation: arm-cut axilla approximation, not the chest tape level.</t>
         </is>
       </c>
     </row>
@@ -2514,13 +2514,13 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Oriented Mesh</t>
+          <t>Arm Vertex Indices, Oriented Mesh</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>_locate_shoulder: take the top ~10% of vertices by z (&gt;= 90th percentile), then the extreme-x vertex (max x = right, min x = left).
-Honest: assumes A-pose. On a T-pose the top-10% band sits at arm height and the extreme-x point lands on the outstretched hand/upper arm, so shoulder, highest-point and wrist collapse together. Pure percentile/extremum, no joint anatomy.</t>
+          <t>_locate_shoulder: shoulder = argmax_z on the segmented arm mesh.
+This replaces whole-body top-10% / extreme-x shoulder selection. It depends on arm segmentation, but prevents head/ear/torso extrema from stealing the shoulder.</t>
         </is>
       </c>
     </row>
@@ -2560,13 +2560,13 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Crotch, Oriented Mesh</t>
+          <t>Crotch, Central Section Geometry</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>_locate_hips: take a horizontal band 5-10% of body height above the crotch, keep faces fully inside the band, split into connected parts and pick the central one (smallest mean |x|), then take its min-x (left) and max-x (right) vertices, snapped to mesh vertices.
-Honest: band fractions hard-coded; finds the widest lateral extent of the torso slab, approximating hip width rather than the anatomical joint.</t>
+          <t>_locate_hips calls hip_section. hip_section scans central horizontal sections above the crotch, rejects off-center loops, smooths depth, and returns the first local depth maximum. Hips are min_x and max_x on that selected pelvis section, snapped to mesh vertices.
+Replaces the fixed 5-10% body-height band above crotch. Remaining risk: abdomen-dominant scans may still need a richer pelvis-transition model.</t>
         </is>
       </c>
     </row>
@@ -2583,13 +2583,13 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Arm Vertex Indices (via Armpits), align_mesh_to_z_axis</t>
+          <t>Arm Vertex Indices, align_mesh_to_z_axis, Stable Section Loop</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>getWrist (Python): align the arm submesh so its long axis is +z, search horizontal slices over 10-30% of arm height (1cm steps), take the centroid of the minimum-perimeter slice, map back via the inverse transform.
-Honest: 'min perimeter' substitutes for the MATLAB min-major-axis. Inherits arm-submesh segmentation, so an A-pose failure propagates here.</t>
+          <t>getWrist (Python): align the arm submesh to +z, sample lower-arm sections, call _stable_wrist_loop, take the centroid of the smallest stable loop, and map back by inverse transform.
+Stability floor = max(0.55*median(perimeters), 0.35*p80(perimeters)); tiny finger/open-boundary slivers are suppressed. Inherits arm-submesh segmentation quality.</t>
         </is>
       </c>
     </row>
@@ -2828,13 +2828,13 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Armpits, Trunk Vertex Indices</t>
+          <t>body_without_arms, Shoulders, Armpits, Section Stack</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Perimeter (section.length) of the trunk cross-section at z = median(armpit_z).
-Honest: raw section perimeter, no convex hull; holes or a non-watertight trunk slice inflate or break the loop.</t>
+          <t>Primary: trunk_girth_levels['chest_full_level']. Build an arm-removed central-section stack and search the shoulder-to-crotch chest band: z = crotch_z + [0.60, 0.78]*(shoulder_z-crotch_z).
+Score chest/bust level from normalized front, depth, perimeter, and area with middle-band bias and axilla-top penalty. If arm removal truncates chest rows, recover from full mesh with lateral x_limit clipping. Measure polygon.exterior.length.</t>
         </is>
       </c>
     </row>
@@ -2851,20 +2851,20 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Armpits, Hips, Trunk Vertex Indices</t>
+          <t>trunk_girth_levels, Section Stack</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Perimeter of the trunk cross-section at z = mean(right_armpit_z, right_hip_z).
-Honest: uses only the right-side landmarks to set the height; not a true narrowest-waist search.</t>
+          <t>Primary: trunk_girth_levels['natural_waist_level']. Natural waist is the area/perimeter/depth narrowing between selected hip and chest levels in the mid torso band.
+Replaces z = mean(right_armpit_z, right_hip_z); no longer right-side-only and no longer a fixed midpoint proxy.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="9">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>hipCircumference</t>
+          <t>stomachPeakCircumference</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -2874,20 +2874,20 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Arm Vertex Indices, Trunk Vertex Indices, Oriented Mesh</t>
+          <t>trunk_girth_levels, Section Stack</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Remove both arms, then take the minimum-perimeter horizontal section over 20 slices in the bottom 10% of trunk height (legs kept).
-Honest: minimum perimeter can pick a slice above the true hip; depends on boolean arm removal succeeding.</t>
+          <t>Primary: trunk_girth_levels['stomach_waist_level']. Select max normalized(front_smooth, perimeter_smooth, area_smooth) between hip and chest.
+Purpose: separate anterior abdomen fullness from natural waist narrowing. Fallback is natural waist measurement.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="9">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>rThighGirth, lThighGirth</t>
+          <t>hipCircumference</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -2897,41 +2897,42 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Hips, Ankle, Leg Vertex Indices</t>
+          <t>body_without_arms, Crotch, Section Stack</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Perimeter of the leg section at z = ankle_z + 0.75*(hip_z - ankle_z), taken in original (un-aligned) coordinates.</t>
+          <t>Primary: trunk_girth_levels['hip_full_level']. Hip curve = normalized(back_smooth, depth_smooth, perimeter_smooth, area_smooth) in the lower pelvis band.
+Targets posterior/depth glute-pelvis fullness rather than global area/width or bottom-trunk minimum perimeter. Fallback: hip_section(no_arms), then slice_measurement.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="9">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>rCalfCircumference, lCalfCircumference</t>
+          <t>rThighGirth, lThighGirth</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Leg Vertex Indices</t>
+          <t>Hips, Ankle, Leg Vertex Indices</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Maximum-perimeter section between 15% and 50% of leg height (leg aligned to +z, ~1in steps).</t>
+          <t>Perimeter of the leg section at z = ankle_z + 0.75*(hip_z - ankle_z), taken in original (un-aligned) coordinates.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="9">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>r_wristgirth, l_wristgirth</t>
+          <t>rCalfCircumference, lCalfCircumference</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -2941,42 +2942,42 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Arm Vertex Indices</t>
+          <t>Leg Vertex Indices</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Minimum section perimeter over 10-30% of arm height - the same slice search as the wrist landmark.</t>
+          <t>Maximum-perimeter section between 15% and 50% of leg height (leg aligned to +z, ~1in steps).</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="9">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>r_forearmgirth, l_forearmgirth</t>
+          <t>r_wristgirth, l_wristgirth</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Arm Vertex Indices</t>
+          <t>Arm Vertex Indices, Stable Section Loop</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Perimeter of the arm section at 50% of arm-submesh height (aligned). The code and the method docstring both use 0.5; an inline code comment still says 25% (stale).
-Honest: this disagrees with the MATLAB spec, which takes the slice at 25% of the wrist-to-armpit axis. Python's 50%-of-segment is a different location and a different reference axis - reconcile before trusting cross-MATLAB parity.</t>
+          <t>Minimum stable lower-arm section perimeter; same _stable_wrist_loop used by the wrist landmark.
+Rejects tiny loops using floor = max(0.55*median(perimeters), 0.35*p80(perimeters)); returns a closed Path3D mapped back to body coordinates.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="9">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>r_bicepgirth, l_bicepgirth</t>
+          <t>r_forearmgirth, l_forearmgirth</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -2991,105 +2992,128 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Perimeter of the arm section at 75% of arm-submesh height (aligned).
-Honest: raw perimeter; the MATLAB note suggests a convex hull at this slice, which Python does not apply.</t>
+          <t>Perimeter of the aligned arm section at 50% of arm-submesh height. Uses shared _arm_section_measurement and _arm_slice_loop; tiny loops are ignored and convex-hull fallback is used only when discrete loops are absent.
+Still differs from MATLAB's 25% wrist-to-armpit reference axis.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="9">
       <c r="A30" s="8" t="inlineStr">
         <is>
+          <t>r_bicepgirth, l_bicepgirth</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Arm Vertex Indices</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Sample aligned arm sections over fractions 0.45..0.62 of arm height; choose the largest clean loop by perimeter and return its closed Path3D.
+Replaces the single fixed 75% slice and reduces sensitivity to local section fragments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="9">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
           <t>r_ankle_girth, l_ankle_girth</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>Leg Vertex Indices</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Minimum section perimeter over the lower 5-25% of leg height (aligned). Slightly wider band than the ankle-landmark search (5-12.5%).</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="9">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32" ht="15" customHeight="1" s="9">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>--- Volume &amp; Surface Area ---</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="n"/>
-      <c r="T31" s="2" t="n"/>
-      <c r="U31" s="2" t="n"/>
-      <c r="V31" s="2" t="n"/>
-      <c r="W31" s="2" t="n"/>
-      <c r="X31" s="2" t="n"/>
-      <c r="Y31" s="2" t="n"/>
-      <c r="Z31" s="2" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="9">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="2" t="n"/>
+      <c r="P32" s="2" t="n"/>
+      <c r="Q32" s="2" t="n"/>
+      <c r="R32" s="2" t="n"/>
+      <c r="S32" s="2" t="n"/>
+      <c r="T32" s="2" t="n"/>
+      <c r="U32" s="2" t="n"/>
+      <c r="V32" s="2" t="n"/>
+      <c r="W32" s="2" t="n"/>
+      <c r="X32" s="2" t="n"/>
+      <c r="Y32" s="2" t="n"/>
+      <c r="Z32" s="2" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="9">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>volume.total, surfaceArea.total</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>Per-part submeshes</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Not implemented as a body-level total. The pipeline never aggregates and main.py prints no volume or area.
 Honest: the per-part trimesh .volume/.area exist (next row) but are never summed; no watertight whole-body volume or area is computed anywhere.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="9">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34" ht="15" customHeight="1" s="9">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>volume (per part), surfaceArea (per part)</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>Part submesh (Arm/Leg/Trunk/Head mesh)</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Each region defines volume/surface_area properties, but they are effectively non-functional.
 Verified on man.obj: Arm and Trunk return self._trimesh.volume/.area and _trimesh is never assigned in src, so left arm, right arm and trunk all raise AttributeError. Leg and Head return self.mesh.volume/.area and run, but give NEGATIVE volumes (head ~ -9.8, each leg ~ -20.85), i.e. inverted/non-watertight results.
@@ -3097,131 +3121,130 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="9">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35" ht="15" customHeight="1" s="9">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>--- Body Segmentation ---</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="n"/>
-      <c r="T34" s="2" t="n"/>
-      <c r="U34" s="2" t="n"/>
-      <c r="V34" s="2" t="n"/>
-      <c r="W34" s="2" t="n"/>
-      <c r="X34" s="2" t="n"/>
-      <c r="Y34" s="2" t="n"/>
-      <c r="Z34" s="2" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="9">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>lArmIdx, rArmIdx</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>Armpits, Oriented Mesh</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>_get_submesh: slice the body at the armpit with a +/-x normal, clean, split into connected parts, keep the part whose highest vertex is largest (the arm).
-Honest: a single planar cut at armpit_x; assumes the arm is the topmost disconnected piece on that side (A-pose). Replaces MATLAB region-growing.</t>
-        </is>
-      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2" t="n"/>
+      <c r="O35" s="2" t="n"/>
+      <c r="P35" s="2" t="n"/>
+      <c r="Q35" s="2" t="n"/>
+      <c r="R35" s="2" t="n"/>
+      <c r="S35" s="2" t="n"/>
+      <c r="T35" s="2" t="n"/>
+      <c r="U35" s="2" t="n"/>
+      <c r="V35" s="2" t="n"/>
+      <c r="W35" s="2" t="n"/>
+      <c r="X35" s="2" t="n"/>
+      <c r="Y35" s="2" t="n"/>
+      <c r="Z35" s="2" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="9">
       <c r="A36" s="8" t="inlineStr">
         <is>
+          <t>lArmIdx, rArmIdx</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Armpits, Oriented Mesh, Crotch, Graph Distances</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>_get_submesh: slice by armpit x-plane, clean, split, reject tiny parts, reject z-span &gt; 0.6*height, reject components below crotch - 0.10*height, then score by outward fraction, z-span, and vertex count.
+If component selection is implausible, geodesic_arm_candidate builds an edge graph, runs Dijkstra from the armpit seed, extracts an arm-like tube, and can replace a connected torso-side slab. Logs vertices and z-range per arm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="9">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
           <t>legIdx</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>Crotch, Hips, Arm Vertex Indices, Oriented Mesh</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>_get_submesh: remove both arms, build a cut plane from the cross product of (hip - crotch) with the front/back axis, slice at the crotch, then slice again on a +/-x plane to keep one side.
 Honest: depends on arm removal and crotch/hip quality; two chained planar slices, no region-grow.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="9">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="38" ht="15" customHeight="1" s="9">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>headIdx</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>Shoulders, Oriented Mesh</t>
         </is>
       </c>
-      <c r="D37" s="11" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>_get_submesh: slice the body above max(shoulder_z), keep the upper part, clean.
 Honest: assumes shoulders are the highest non-head points and that a single horizontal cut separates the head.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="9">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39" ht="15.75" customHeight="1" s="9">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>trunkIdx</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Hard</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Leg Vertex Indices, Arm Vertex Indices, Head Vertex Indices</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>_get_submesh: boolean-difference the body minus both legs, both arms, and the head.
 Honest: 'trunk = body - everything else', so correctness is bounded by every other segmentation and by boolean-op robustness on imperfect meshes.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1" s="9"/>
     <row r="40" ht="15.75" customHeight="1" s="9"/>
     <row r="41" ht="15.75" customHeight="1" s="9"/>
     <row r="42" ht="15.75" customHeight="1" s="9"/>

</xml_diff>